<commit_message>
Dash DI - 19/09/2026
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -34,13 +34,13 @@
     <t>COD_XP</t>
   </si>
   <si>
-    <t>CDB</t>
-  </si>
-  <si>
-    <t>CDB3251WXH0</t>
-  </si>
-  <si>
-    <t>REAL FIM</t>
+    <t>LFSN</t>
+  </si>
+  <si>
+    <t>LFSN19001BC</t>
+  </si>
+  <si>
+    <t>FIRF GERAES 30</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="2">
-        <v>46454</v>
+        <v>46486</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>

</xml_diff>